<commit_message>
Complete Task 2 and updated checklist
</commit_message>
<xml_diff>
--- a/checklist.xlsx
+++ b/checklist.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="260">
   <si>
     <t>iNeuBytes  •  45-Day Web Development Internship  -  Intern Checklist</t>
   </si>
@@ -324,112 +324,151 @@
     <t>9</t>
   </si>
   <si>
+    <t>Created HealSphere appointment-booking landing page with navbar, hero section, CTA, and navigation to key sections.</t>
+  </si>
+  <si>
+    <t>HTML: Doctor Listing page</t>
+  </si>
+  <si>
+    <t>Grid/list of doctors</t>
+  </si>
+  <si>
+    <t>9-10</t>
+  </si>
+  <si>
+    <t>Added six doctor cards with doctor name, qualification, specialization, experience, consultation fee, availability, and profile buttons.</t>
+  </si>
+  <si>
+    <t>HTML: Doctor Details / Profile page</t>
+  </si>
+  <si>
+    <t>Name, Department, Experience, Available Time Slots, Consultation Fee</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Added doctor profile section with placeholder content, dynamically populated by JavaScript with department, qualification, experience, fee, availability, and description.</t>
+  </si>
+  <si>
+    <t>HTML: Appointment Booking form</t>
+  </si>
+  <si>
+    <t>Select Doctor, Select Date, Select Time Slot, Patient Details, Book</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>Created booking form with patient details, doctor dropdown, date selection, time-slot buttons, reason for visit, and confirmation button.</t>
+  </si>
+  <si>
+    <t>HTML: Confirmation &amp; Summary/History</t>
+  </si>
+  <si>
+    <t>Appointment confirmation + appointment summary (frontend)</t>
+  </si>
+  <si>
+    <t>Added appointment summary and appointment-history sections with containers for dynamically generated booking information.</t>
+  </si>
+  <si>
+    <t>CSS: responsive layout &amp; cards</t>
+  </si>
+  <si>
+    <t>Doctor profile cards, booking forms, buttons, nav - professional theme</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>Implemented professional healthcare styling with responsive layouts, doctor cards, forms, buttons, hover effects, mobile menu styling, and tablet/mobile breakpoints.</t>
+  </si>
+  <si>
+    <t>JS: doctor search &amp; department filter</t>
+  </si>
+  <si>
+    <t>Search by name; filter by department</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>Implemented live doctor-name search and department filtering using data-name and data-department attributes.</t>
+  </si>
+  <si>
+    <t>JS: appointment booking + validation</t>
+  </si>
+  <si>
+    <t>Booking flow, form validation, dynamic appointment summary</t>
+  </si>
+  <si>
+    <t>13-14</t>
+  </si>
+  <si>
+    <t>Implemented booking workflow, patient/email/phone/date/time/message validation, dynamic appointment object creation, confirmation summary, and form reset.</t>
+  </si>
+  <si>
+    <t>JS: local storage (optional)</t>
+  </si>
+  <si>
+    <t>Persist appointments on the frontend</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>Implemented browser localStorage persistence using JSON stringify/parse so appointments remain available after page reload.</t>
+  </si>
+  <si>
+    <t>Booking workflow, responsiveness, search/filters, forms, cross-browser</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>Verified doctor search/filtering, profile generation, appointment validation, time-slot selection, summary/history updates, responsive layouts, and navigation functionality.</t>
+  </si>
+  <si>
+    <t>Push Task 2 to GitHub</t>
+  </si>
+  <si>
+    <t>Commit into the Task 2 folder</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>Task 2 files are complete locally, committed and pushed to the Github Task-2 folder.</t>
+  </si>
+  <si>
+    <t>Write Task 2 development report</t>
+  </si>
+  <si>
+    <t>Detailed write-up in the Google Doc</t>
+  </si>
+  <si>
+    <t>Documented the Task 2 development approach, features, technologies, functionality, and results in the Google Doc.</t>
+  </si>
+  <si>
+    <t>Project demonstration walkthrough</t>
+  </si>
+  <si>
+    <t>Recorded a walkthrough demonstrating the Doctor Appointment Booking System and its major features.</t>
+  </si>
+  <si>
+    <t>3 · Task 3 - Healthcare Management Dashboard</t>
+  </si>
+  <si>
+    <t>HTML: Dashboard shell</t>
+  </si>
+  <si>
+    <t>Dashboard Home, sidebar navigation, top navigation bar, user profile section</t>
+  </si>
+  <si>
+    <t>17-18</t>
+  </si>
+  <si>
     <t>Not Started</t>
-  </si>
-  <si>
-    <t>HTML: Doctor Listing page</t>
-  </si>
-  <si>
-    <t>Grid/list of doctors</t>
-  </si>
-  <si>
-    <t>9-10</t>
-  </si>
-  <si>
-    <t>HTML: Doctor Details / Profile page</t>
-  </si>
-  <si>
-    <t>Name, Department, Experience, Available Time Slots, Consultation Fee</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>HTML: Appointment Booking form</t>
-  </si>
-  <si>
-    <t>Select Doctor, Select Date, Select Time Slot, Patient Details, Book</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>HTML: Confirmation &amp; Summary/History</t>
-  </si>
-  <si>
-    <t>Appointment confirmation + appointment summary (frontend)</t>
-  </si>
-  <si>
-    <t>CSS: responsive layout &amp; cards</t>
-  </si>
-  <si>
-    <t>Doctor profile cards, booking forms, buttons, nav - professional theme</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>JS: doctor search &amp; department filter</t>
-  </si>
-  <si>
-    <t>Search by name; filter by department</t>
-  </si>
-  <si>
-    <t>13</t>
-  </si>
-  <si>
-    <t>JS: appointment booking + validation</t>
-  </si>
-  <si>
-    <t>Booking flow, form validation, dynamic appointment summary</t>
-  </si>
-  <si>
-    <t>13-14</t>
-  </si>
-  <si>
-    <t>JS: local storage (optional)</t>
-  </si>
-  <si>
-    <t>Persist appointments on the frontend</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>Booking workflow, responsiveness, search/filters, forms, cross-browser</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>Push Task 2 to GitHub</t>
-  </si>
-  <si>
-    <t>Commit into the Task 2 folder</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>Write Task 2 development report</t>
-  </si>
-  <si>
-    <t>Detailed write-up in the Google Doc</t>
-  </si>
-  <si>
-    <t>Project demonstration walkthrough</t>
-  </si>
-  <si>
-    <t>3 · Task 3 - Healthcare Management Dashboard</t>
-  </si>
-  <si>
-    <t>HTML: Dashboard shell</t>
-  </si>
-  <si>
-    <t>Dashboard Home, sidebar navigation, top navigation bar, user profile section</t>
-  </si>
-  <si>
-    <t>17-18</t>
   </si>
   <si>
     <t>HTML: Doctor Management page</t>
@@ -1512,7 +1551,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1569,9 +1608,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1978,8 +2014,8 @@
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
       <c r="D4" s="7" t="str">
-        <f>"24 of 78 done   ("&amp;TEXT(24/78,"0%")&amp;" complete)   |   In Progress: 1   |   Blocked: 0"</f>
-        <v>24 of 78 done   (31% complete)   |   In Progress: 1   |   Blocked: 0</v>
+        <f>"37 of 78 done   ("&amp;TEXT(37/78,"0%")&amp;" complete)   |   In Progress: 1   |   Blocked: 0"</f>
+        <v>37 of 78 done   (47% complete)   |   In Progress: 1   |   Blocked: 0</v>
       </c>
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
@@ -2495,7 +2531,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="30" ht="30" customHeight="1" spans="1:7">
+    <row r="30" ht="31" customHeight="1" spans="1:7">
       <c r="A30" s="14">
         <v>24</v>
       </c>
@@ -2533,9 +2569,11 @@
         <v>97</v>
       </c>
       <c r="F31" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G31" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="G31" s="20"/>
     </row>
     <row r="32" ht="30" customHeight="1" spans="1:7">
       <c r="A32" s="14">
@@ -2551,10 +2589,12 @@
       <c r="E32" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="F32" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="G32" s="17"/>
+      <c r="F32" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G32" s="17" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="33" ht="30" customHeight="1" spans="1:7">
       <c r="A33" s="9">
@@ -2562,18 +2602,20 @@
       </c>
       <c r="B33" s="10"/>
       <c r="C33" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F33" s="13" t="s">
-        <v>98</v>
-      </c>
-      <c r="G33" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G33" s="12" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="34" ht="30" customHeight="1" spans="1:7">
       <c r="A34" s="14">
@@ -2581,18 +2623,20 @@
       </c>
       <c r="B34" s="15"/>
       <c r="C34" s="16" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D34" s="17" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E34" s="18" t="s">
-        <v>107</v>
-      </c>
-      <c r="F34" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="G34" s="17"/>
+        <v>109</v>
+      </c>
+      <c r="F34" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G34" s="17" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="35" ht="30" customHeight="1" spans="1:7">
       <c r="A35" s="9">
@@ -2600,18 +2644,20 @@
       </c>
       <c r="B35" s="10"/>
       <c r="C35" s="11" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D35" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="E35" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="E35" s="13" t="s">
-        <v>107</v>
-      </c>
       <c r="F35" s="13" t="s">
-        <v>98</v>
-      </c>
-      <c r="G35" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G35" s="12" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="36" ht="30" customHeight="1" spans="1:7">
       <c r="A36" s="14">
@@ -2619,18 +2665,20 @@
       </c>
       <c r="B36" s="15"/>
       <c r="C36" s="16" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="D36" s="17" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="E36" s="18" t="s">
-        <v>112</v>
-      </c>
-      <c r="F36" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="G36" s="17"/>
+        <v>116</v>
+      </c>
+      <c r="F36" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G36" s="17" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="37" ht="30" customHeight="1" spans="1:7">
       <c r="A37" s="9">
@@ -2638,18 +2686,20 @@
       </c>
       <c r="B37" s="10"/>
       <c r="C37" s="11" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="F37" s="13" t="s">
-        <v>98</v>
-      </c>
-      <c r="G37" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G37" s="12" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="38" ht="30" customHeight="1" spans="1:7">
       <c r="A38" s="14">
@@ -2657,18 +2707,20 @@
       </c>
       <c r="B38" s="15"/>
       <c r="C38" s="16" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="D38" s="17" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="E38" s="18" t="s">
-        <v>118</v>
-      </c>
-      <c r="F38" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="G38" s="17"/>
+        <v>124</v>
+      </c>
+      <c r="F38" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G38" s="17" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="39" ht="30" customHeight="1" spans="1:7">
       <c r="A39" s="9">
@@ -2676,18 +2728,20 @@
       </c>
       <c r="B39" s="10"/>
       <c r="C39" s="11" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="E39" s="13" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="F39" s="13" t="s">
-        <v>98</v>
-      </c>
-      <c r="G39" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G39" s="12" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="40" ht="30" customHeight="1" spans="1:7">
       <c r="A40" s="14">
@@ -2698,15 +2752,17 @@
         <v>81</v>
       </c>
       <c r="D40" s="17" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="E40" s="18" t="s">
-        <v>123</v>
-      </c>
-      <c r="F40" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="G40" s="17"/>
+        <v>131</v>
+      </c>
+      <c r="F40" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G40" s="17" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="41" ht="30" customHeight="1" spans="1:7">
       <c r="A41" s="9">
@@ -2714,18 +2770,20 @@
       </c>
       <c r="B41" s="10"/>
       <c r="C41" s="11" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="E41" s="13" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="F41" s="13" t="s">
-        <v>98</v>
-      </c>
-      <c r="G41" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G41" s="12" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="42" ht="30" customHeight="1" spans="1:7">
       <c r="A42" s="14">
@@ -2733,18 +2791,20 @@
       </c>
       <c r="B42" s="15"/>
       <c r="C42" s="16" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="D42" s="17" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="E42" s="18" t="s">
-        <v>126</v>
-      </c>
-      <c r="F42" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="G42" s="17"/>
+        <v>135</v>
+      </c>
+      <c r="F42" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G42" s="17" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="43" ht="30" customHeight="1" spans="1:7">
       <c r="A43" s="9">
@@ -2755,34 +2815,36 @@
         <v>91</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="E43" s="13" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="F43" s="13" t="s">
-        <v>98</v>
-      </c>
-      <c r="G43" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G43" s="12" t="s">
+        <v>141</v>
+      </c>
     </row>
     <row r="44" ht="30" customHeight="1" spans="1:7">
       <c r="A44" s="14">
         <v>38</v>
       </c>
       <c r="B44" s="15" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="D44" s="17" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="E44" s="18" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="F44" s="18" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G44" s="17"/>
     </row>
@@ -2792,16 +2854,16 @@
       </c>
       <c r="B45" s="10"/>
       <c r="C45" s="11" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="D45" s="12" t="s">
-        <v>135</v>
+        <v>148</v>
       </c>
       <c r="E45" s="13" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="F45" s="13" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G45" s="12"/>
     </row>
@@ -2811,16 +2873,16 @@
       </c>
       <c r="B46" s="15"/>
       <c r="C46" s="16" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
       <c r="D46" s="17" t="s">
-        <v>135</v>
+        <v>148</v>
       </c>
       <c r="E46" s="18" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="F46" s="18" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G46" s="17"/>
     </row>
@@ -2830,16 +2892,16 @@
       </c>
       <c r="B47" s="10"/>
       <c r="C47" s="11" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="D47" s="12" t="s">
-        <v>139</v>
+        <v>152</v>
       </c>
       <c r="E47" s="13" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="F47" s="13" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G47" s="12"/>
     </row>
@@ -2849,16 +2911,16 @@
       </c>
       <c r="B48" s="15"/>
       <c r="C48" s="16" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="D48" s="17" t="s">
-        <v>142</v>
+        <v>155</v>
       </c>
       <c r="E48" s="18" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="F48" s="18" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G48" s="17"/>
     </row>
@@ -2868,16 +2930,16 @@
       </c>
       <c r="B49" s="10"/>
       <c r="C49" s="11" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
       <c r="D49" s="12" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="E49" s="13" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="F49" s="13" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G49" s="12"/>
     </row>
@@ -2887,16 +2949,16 @@
       </c>
       <c r="B50" s="15"/>
       <c r="C50" s="16" t="s">
-        <v>145</v>
+        <v>158</v>
       </c>
       <c r="D50" s="17" t="s">
-        <v>146</v>
+        <v>159</v>
       </c>
       <c r="E50" s="18" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="F50" s="18" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G50" s="17"/>
     </row>
@@ -2906,16 +2968,16 @@
       </c>
       <c r="B51" s="10"/>
       <c r="C51" s="11" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="D51" s="12" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="E51" s="13" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="F51" s="13" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G51" s="12"/>
     </row>
@@ -2925,16 +2987,16 @@
       </c>
       <c r="B52" s="15"/>
       <c r="C52" s="16" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
       <c r="D52" s="17" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="E52" s="18" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="F52" s="18" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -2944,16 +3006,16 @@
       </c>
       <c r="B53" s="10"/>
       <c r="C53" s="11" t="s">
-        <v>153</v>
+        <v>166</v>
       </c>
       <c r="D53" s="12" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
       <c r="E53" s="13" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
       <c r="F53" s="13" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G53" s="12"/>
     </row>
@@ -2963,16 +3025,16 @@
       </c>
       <c r="B54" s="15"/>
       <c r="C54" s="16" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="D54" s="17" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="E54" s="18" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
       <c r="F54" s="18" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G54" s="17"/>
     </row>
@@ -2982,16 +3044,16 @@
       </c>
       <c r="B55" s="10"/>
       <c r="C55" s="11" t="s">
-        <v>158</v>
+        <v>171</v>
       </c>
       <c r="D55" s="12" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="E55" s="13" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="F55" s="13" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G55" s="12"/>
     </row>
@@ -3004,13 +3066,13 @@
         <v>77</v>
       </c>
       <c r="D56" s="17" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
       <c r="E56" s="18" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="F56" s="18" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G56" s="17"/>
     </row>
@@ -3023,13 +3085,13 @@
         <v>81</v>
       </c>
       <c r="D57" s="12" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="E57" s="13" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="F57" s="13" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G57" s="12"/>
     </row>
@@ -3039,16 +3101,16 @@
       </c>
       <c r="B58" s="15"/>
       <c r="C58" s="16" t="s">
-        <v>163</v>
+        <v>176</v>
       </c>
       <c r="D58" s="17" t="s">
-        <v>164</v>
+        <v>177</v>
       </c>
       <c r="E58" s="18" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="F58" s="18" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G58" s="17"/>
     </row>
@@ -3058,16 +3120,16 @@
       </c>
       <c r="B59" s="10"/>
       <c r="C59" s="11" t="s">
-        <v>166</v>
+        <v>179</v>
       </c>
       <c r="D59" s="12" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="E59" s="13" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="F59" s="13" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G59" s="12"/>
     </row>
@@ -3080,13 +3142,13 @@
         <v>91</v>
       </c>
       <c r="D60" s="17" t="s">
-        <v>168</v>
+        <v>181</v>
       </c>
       <c r="E60" s="18" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="F60" s="18" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G60" s="17"/>
     </row>
@@ -3095,19 +3157,19 @@
         <v>55</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="C61" s="11" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
       <c r="D61" s="12" t="s">
-        <v>171</v>
+        <v>184</v>
       </c>
       <c r="E61" s="13" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="F61" s="13" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G61" s="12"/>
     </row>
@@ -3117,16 +3179,16 @@
       </c>
       <c r="B62" s="15"/>
       <c r="C62" s="16" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="D62" s="17" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
       <c r="E62" s="18" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="F62" s="18" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G62" s="17"/>
     </row>
@@ -3136,16 +3198,16 @@
       </c>
       <c r="B63" s="10"/>
       <c r="C63" s="11" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="D63" s="12" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="E63" s="13" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="F63" s="13" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G63" s="12"/>
     </row>
@@ -3155,16 +3217,16 @@
       </c>
       <c r="B64" s="15"/>
       <c r="C64" s="16" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="D64" s="17" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="E64" s="18" t="s">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="F64" s="18" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G64" s="17"/>
     </row>
@@ -3174,16 +3236,16 @@
       </c>
       <c r="B65" s="10"/>
       <c r="C65" s="11" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="D65" s="12" t="s">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="E65" s="13" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
       <c r="F65" s="13" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G65" s="12"/>
     </row>
@@ -3193,16 +3255,16 @@
       </c>
       <c r="B66" s="15"/>
       <c r="C66" s="16" t="s">
-        <v>185</v>
+        <v>198</v>
       </c>
       <c r="D66" s="17" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="E66" s="18" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="F66" s="18" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G66" s="17"/>
     </row>
@@ -3212,16 +3274,16 @@
       </c>
       <c r="B67" s="10"/>
       <c r="C67" s="11" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="D67" s="12" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="E67" s="13" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
       <c r="F67" s="13" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G67" s="12"/>
     </row>
@@ -3231,16 +3293,16 @@
       </c>
       <c r="B68" s="15"/>
       <c r="C68" s="16" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="D68" s="17" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="E68" s="18" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="F68" s="18" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G68" s="17"/>
     </row>
@@ -3250,16 +3312,16 @@
       </c>
       <c r="B69" s="10"/>
       <c r="C69" s="11" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="D69" s="12" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="E69" s="13" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="F69" s="13" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G69" s="12"/>
     </row>
@@ -3269,16 +3331,16 @@
       </c>
       <c r="B70" s="15"/>
       <c r="C70" s="16" t="s">
-        <v>197</v>
+        <v>210</v>
       </c>
       <c r="D70" s="17" t="s">
-        <v>198</v>
+        <v>211</v>
       </c>
       <c r="E70" s="18" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="F70" s="18" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G70" s="17"/>
     </row>
@@ -3288,16 +3350,16 @@
       </c>
       <c r="B71" s="10"/>
       <c r="C71" s="11" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
       <c r="D71" s="12" t="s">
-        <v>201</v>
+        <v>214</v>
       </c>
       <c r="E71" s="13" t="s">
-        <v>202</v>
+        <v>215</v>
       </c>
       <c r="F71" s="13" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G71" s="12"/>
     </row>
@@ -3307,16 +3369,16 @@
       </c>
       <c r="B72" s="15"/>
       <c r="C72" s="16" t="s">
-        <v>203</v>
+        <v>216</v>
       </c>
       <c r="D72" s="17" t="s">
-        <v>204</v>
+        <v>217</v>
       </c>
       <c r="E72" s="18" t="s">
-        <v>202</v>
+        <v>215</v>
       </c>
       <c r="F72" s="18" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G72" s="17"/>
     </row>
@@ -3326,16 +3388,16 @@
       </c>
       <c r="B73" s="10"/>
       <c r="C73" s="11" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="D73" s="12" t="s">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="E73" s="13" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="F73" s="13" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G73" s="12"/>
     </row>
@@ -3345,16 +3407,16 @@
       </c>
       <c r="B74" s="15"/>
       <c r="C74" s="16" t="s">
-        <v>208</v>
+        <v>221</v>
       </c>
       <c r="D74" s="17" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
       <c r="E74" s="18" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="F74" s="18" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G74" s="17"/>
     </row>
@@ -3364,16 +3426,16 @@
       </c>
       <c r="B75" s="10"/>
       <c r="C75" s="11" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="D75" s="12" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
       <c r="E75" s="13" t="s">
-        <v>212</v>
+        <v>225</v>
       </c>
       <c r="F75" s="13" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G75" s="12"/>
     </row>
@@ -3383,16 +3445,16 @@
       </c>
       <c r="B76" s="15"/>
       <c r="C76" s="16" t="s">
-        <v>213</v>
+        <v>226</v>
       </c>
       <c r="D76" s="17" t="s">
-        <v>214</v>
+        <v>227</v>
       </c>
       <c r="E76" s="18" t="s">
-        <v>212</v>
+        <v>225</v>
       </c>
       <c r="F76" s="18" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G76" s="17"/>
     </row>
@@ -3402,16 +3464,16 @@
       </c>
       <c r="B77" s="10"/>
       <c r="C77" s="11" t="s">
-        <v>215</v>
+        <v>228</v>
       </c>
       <c r="D77" s="12" t="s">
-        <v>216</v>
+        <v>229</v>
       </c>
       <c r="E77" s="13" t="s">
-        <v>212</v>
+        <v>225</v>
       </c>
       <c r="F77" s="13" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G77" s="12"/>
     </row>
@@ -3421,16 +3483,16 @@
       </c>
       <c r="B78" s="15"/>
       <c r="C78" s="16" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="D78" s="17" t="s">
-        <v>218</v>
+        <v>231</v>
       </c>
       <c r="E78" s="18" t="s">
-        <v>219</v>
+        <v>232</v>
       </c>
       <c r="F78" s="18" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G78" s="17"/>
     </row>
@@ -3440,16 +3502,16 @@
       </c>
       <c r="B79" s="10"/>
       <c r="C79" s="11" t="s">
-        <v>220</v>
+        <v>233</v>
       </c>
       <c r="D79" s="12" t="s">
-        <v>221</v>
+        <v>234</v>
       </c>
       <c r="E79" s="13" t="s">
-        <v>219</v>
+        <v>232</v>
       </c>
       <c r="F79" s="13" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G79" s="12"/>
     </row>
@@ -3459,16 +3521,16 @@
       </c>
       <c r="B80" s="15"/>
       <c r="C80" s="16" t="s">
-        <v>222</v>
+        <v>235</v>
       </c>
       <c r="D80" s="17" t="s">
-        <v>223</v>
+        <v>236</v>
       </c>
       <c r="E80" s="18" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="F80" s="18" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G80" s="17"/>
     </row>
@@ -3478,16 +3540,16 @@
       </c>
       <c r="B81" s="10"/>
       <c r="C81" s="11" t="s">
-        <v>225</v>
+        <v>238</v>
       </c>
       <c r="D81" s="12" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="E81" s="13" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="F81" s="13" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G81" s="12"/>
     </row>
@@ -3497,16 +3559,16 @@
       </c>
       <c r="B82" s="15"/>
       <c r="C82" s="16" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
       <c r="D82" s="17" t="s">
-        <v>228</v>
+        <v>241</v>
       </c>
       <c r="E82" s="18" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="F82" s="18" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G82" s="17"/>
     </row>
@@ -3516,16 +3578,16 @@
       </c>
       <c r="B83" s="10"/>
       <c r="C83" s="11" t="s">
-        <v>229</v>
+        <v>242</v>
       </c>
       <c r="D83" s="12" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="E83" s="13" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="F83" s="13" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G83" s="12"/>
     </row>
@@ -3535,16 +3597,16 @@
       </c>
       <c r="B84" s="10"/>
       <c r="C84" s="11" t="s">
-        <v>231</v>
+        <v>244</v>
       </c>
       <c r="D84" s="12" t="s">
-        <v>232</v>
+        <v>245</v>
       </c>
       <c r="E84" s="13" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="F84" s="13" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="G84" s="12"/>
     </row>
@@ -3568,7 +3630,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F7:F30 F31:F84">
+    <dataValidation type="list" allowBlank="1" sqref="F7:F29 F30:F43 F44:F84">
       <formula1>"Not Started,In Progress,Done,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3590,73 +3652,73 @@
   <sheetData>
     <row r="1" ht="27.75" customHeight="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>233</v>
+        <v>246</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="3" ht="30" customHeight="1" spans="2:2">
       <c r="B3" s="2" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="2:2">
       <c r="B4" s="2" t="s">
-        <v>235</v>
+        <v>248</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="2:2">
       <c r="B5" s="2" t="s">
-        <v>236</v>
+        <v>249</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="2:2">
       <c r="B6" s="2" t="s">
-        <v>237</v>
+        <v>250</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="2:2">
       <c r="B7" s="2" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" spans="2:2">
       <c r="B8" s="2" t="s">
-        <v>239</v>
+        <v>252</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" spans="2:2">
       <c r="B9" s="2" t="s">
-        <v>240</v>
+        <v>253</v>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1" spans="2:2">
       <c r="B10" s="2" t="s">
-        <v>241</v>
+        <v>254</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1" spans="2:2">
       <c r="B11" s="2" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1" spans="2:2">
       <c r="B12" s="2" t="s">
-        <v>243</v>
+        <v>256</v>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1" spans="2:2">
       <c r="B13" s="2" t="s">
-        <v>244</v>
+        <v>257</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1" spans="2:2">
       <c r="B14" s="2" t="s">
-        <v>245</v>
+        <v>258</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1" spans="2:2">
       <c r="B15" s="2" t="s">
-        <v>246</v>
+        <v>259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Complete Task 3 and updated checklist
</commit_message>
<xml_diff>
--- a/checklist.xlsx
+++ b/checklist.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="276">
   <si>
     <t>iNeuBytes  •  45-Day Web Development Internship  -  Intern Checklist</t>
   </si>
@@ -468,124 +468,172 @@
     <t>17-18</t>
   </si>
   <si>
+    <t>Dashboard, sidebar navigation, top navigation and admin profile implemented.</t>
+  </si>
+  <si>
+    <t>HTML: Doctor Management page</t>
+  </si>
+  <si>
+    <t>Table + add/edit/delete/search controls</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>Doctor table with add, edit, delete and search controls implemented.</t>
+  </si>
+  <si>
+    <t>HTML: Patient Management page</t>
+  </si>
+  <si>
+    <t>Patient table with add, edit, delete and search controls implemented.</t>
+  </si>
+  <si>
+    <t>HTML: Appointment Management page</t>
+  </si>
+  <si>
+    <t>Table + search, filter by status, update status</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>Appointment table with search, status filter and status update controls implemented.</t>
+  </si>
+  <si>
+    <t>HTML: Department Management page</t>
+  </si>
+  <si>
+    <t>Table + add/edit/delete controls</t>
+  </si>
+  <si>
+    <t>Department table with add, edit and delete controls implemented.</t>
+  </si>
+  <si>
+    <t>Statistics cards</t>
+  </si>
+  <si>
+    <t>Total Doctors, Total Patients, Total Appointments, Department statistics</t>
+  </si>
+  <si>
+    <t>Dynamic doctor, patient, appointment and department statistics displayed.</t>
+  </si>
+  <si>
+    <t>CSS: dashboard styling</t>
+  </si>
+  <si>
+    <t>Dashboard layout, sidebar, responsive tables, cards, buttons, forms - professional admin UI</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>Responsive admin dashboard UI with sidebar, cards, tables, forms and buttons styled.</t>
+  </si>
+  <si>
+    <t>JS: Doctor CRUD (Local Storage)</t>
+  </si>
+  <si>
+    <t>View, Add, Edit, Delete, Search doctors</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>Doctor data persisted with Local Storage; add, edit, delete and search tested.</t>
+  </si>
+  <si>
+    <t>JS: Patient CRUD (Local Storage)</t>
+  </si>
+  <si>
+    <t>View, Add, Edit, Delete, Search patients</t>
+  </si>
+  <si>
+    <t>Patient data persisted with Local Storage; add, edit, delete and search tested.</t>
+  </si>
+  <si>
+    <t>JS: Appointment management</t>
+  </si>
+  <si>
+    <t>View, search, filter by status, update appointment status</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>Appointment viewing, search, status filtering, status updates and persistence tested.</t>
+  </si>
+  <si>
+    <t>JS: Department CRUD</t>
+  </si>
+  <si>
+    <t>View, Add, Edit, Delete departments</t>
+  </si>
+  <si>
+    <t>Department add, edit and delete operations tested with Local Storage.</t>
+  </si>
+  <si>
+    <t>JS: dynamic statistics &amp; tables</t>
+  </si>
+  <si>
+    <t>Dynamic dashboard stats, filtering, table manipulation, form validation</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>Dashboard statistics and management tables update dynamically after data changes.</t>
+  </si>
+  <si>
+    <t>Mobile, tablet, desktop responsive dashboard</t>
+  </si>
+  <si>
+    <t>Dashboard tested successfully at desktop, tablet and mobile resolutions.</t>
+  </si>
+  <si>
+    <t>Verify CRUD, responsiveness, forms, cross-browser; fix UI/functionality issues</t>
+  </si>
+  <si>
+    <t>CRUD, search/filtering, persistence, responsiveness and console errors tested; no red console errors found.</t>
+  </si>
+  <si>
+    <t>Push Task 3 to GitHub</t>
+  </si>
+  <si>
+    <t>Commit into the Task 3 folder</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>Task 3 and updated checklist committed and pushed to the public repository.</t>
+  </si>
+  <si>
+    <t>Write Task 3 development report</t>
+  </si>
+  <si>
+    <t>Document in the Google Doc</t>
+  </si>
+  <si>
+    <t>Task 3 development report documented in the Google Doc.</t>
+  </si>
+  <si>
+    <t>Dashboard demonstration</t>
+  </si>
+  <si>
+    <t>4 · Major Project - Healthcare / Clinic Management System</t>
+  </si>
+  <si>
+    <t>Auth: registration &amp; login</t>
+  </si>
+  <si>
+    <t>Secure sign-up/login; separate login for Patient, Doctor, Admin</t>
+  </si>
+  <si>
+    <t>25-26</t>
+  </si>
+  <si>
     <t>Not Started</t>
-  </si>
-  <si>
-    <t>HTML: Doctor Management page</t>
-  </si>
-  <si>
-    <t>Table + add/edit/delete/search controls</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>HTML: Patient Management page</t>
-  </si>
-  <si>
-    <t>HTML: Appointment Management page</t>
-  </si>
-  <si>
-    <t>Table + search, filter by status, update status</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>HTML: Department Management page</t>
-  </si>
-  <si>
-    <t>Table + add/edit/delete controls</t>
-  </si>
-  <si>
-    <t>Statistics cards</t>
-  </si>
-  <si>
-    <t>Total Doctors, Total Patients, Total Appointments, Department statistics</t>
-  </si>
-  <si>
-    <t>CSS: dashboard styling</t>
-  </si>
-  <si>
-    <t>Dashboard layout, sidebar, responsive tables, cards, buttons, forms - professional admin UI</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>JS: Doctor CRUD (Local Storage)</t>
-  </si>
-  <si>
-    <t>View, Add, Edit, Delete, Search doctors</t>
-  </si>
-  <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>JS: Patient CRUD (Local Storage)</t>
-  </si>
-  <si>
-    <t>View, Add, Edit, Delete, Search patients</t>
-  </si>
-  <si>
-    <t>JS: Appointment management</t>
-  </si>
-  <si>
-    <t>View, search, filter by status, update appointment status</t>
-  </si>
-  <si>
-    <t>22</t>
-  </si>
-  <si>
-    <t>JS: Department CRUD</t>
-  </si>
-  <si>
-    <t>View, Add, Edit, Delete departments</t>
-  </si>
-  <si>
-    <t>JS: dynamic statistics &amp; tables</t>
-  </si>
-  <si>
-    <t>Dynamic dashboard stats, filtering, table manipulation, form validation</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
-    <t>Mobile, tablet, desktop responsive dashboard</t>
-  </si>
-  <si>
-    <t>Verify CRUD, responsiveness, forms, cross-browser; fix UI/functionality issues</t>
-  </si>
-  <si>
-    <t>Push Task 3 to GitHub</t>
-  </si>
-  <si>
-    <t>Commit into the Task 3 folder</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>Write Task 3 development report</t>
-  </si>
-  <si>
-    <t>Document in the Google Doc</t>
-  </si>
-  <si>
-    <t>Dashboard demonstration</t>
-  </si>
-  <si>
-    <t>4 · Major Project - Healthcare / Clinic Management System</t>
-  </si>
-  <si>
-    <t>Auth: registration &amp; login</t>
-  </si>
-  <si>
-    <t>Secure sign-up/login; separate login for Patient, Doctor, Admin</t>
-  </si>
-  <si>
-    <t>25-26</t>
   </si>
   <si>
     <t>Auth: role-based access control</t>
@@ -2014,8 +2062,8 @@
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
       <c r="D4" s="7" t="str">
-        <f>"37 of 78 done   ("&amp;TEXT(37/78,"0%")&amp;" complete)   |   In Progress: 1   |   Blocked: 0"</f>
-        <v>37 of 78 done   (47% complete)   |   In Progress: 1   |   Blocked: 0</v>
+        <f>"54 of 78 done   ("&amp;TEXT(54/78,"0%")&amp;" complete)   |   In Progress: 1   |   Blocked: 0"</f>
+        <v>54 of 78 done   (69% complete)   |   In Progress: 1   |   Blocked: 0</v>
       </c>
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
@@ -2843,10 +2891,12 @@
       <c r="E44" s="18" t="s">
         <v>145</v>
       </c>
-      <c r="F44" s="18" t="s">
+      <c r="F44" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G44" s="17" t="s">
         <v>146</v>
       </c>
-      <c r="G44" s="17"/>
     </row>
     <row r="45" ht="30" customHeight="1" spans="1:7">
       <c r="A45" s="9">
@@ -2863,9 +2913,11 @@
         <v>149</v>
       </c>
       <c r="F45" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="G45" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G45" s="12" t="s">
+        <v>150</v>
+      </c>
     </row>
     <row r="46" ht="30" customHeight="1" spans="1:7">
       <c r="A46" s="14">
@@ -2873,7 +2925,7 @@
       </c>
       <c r="B46" s="15"/>
       <c r="C46" s="16" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D46" s="17" t="s">
         <v>148</v>
@@ -2881,10 +2933,12 @@
       <c r="E46" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="F46" s="18" t="s">
-        <v>146</v>
-      </c>
-      <c r="G46" s="17"/>
+      <c r="F46" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G46" s="17" t="s">
+        <v>152</v>
+      </c>
     </row>
     <row r="47" ht="30" customHeight="1" spans="1:7">
       <c r="A47" s="9">
@@ -2892,18 +2946,20 @@
       </c>
       <c r="B47" s="10"/>
       <c r="C47" s="11" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D47" s="12" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E47" s="13" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="F47" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="G47" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G47" s="12" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="48" ht="30" customHeight="1" spans="1:7">
       <c r="A48" s="14">
@@ -2911,18 +2967,20 @@
       </c>
       <c r="B48" s="15"/>
       <c r="C48" s="16" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="D48" s="17" t="s">
+        <v>158</v>
+      </c>
+      <c r="E48" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="E48" s="18" t="s">
-        <v>153</v>
-      </c>
-      <c r="F48" s="18" t="s">
-        <v>146</v>
-      </c>
-      <c r="G48" s="17"/>
+      <c r="F48" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G48" s="17" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="49" ht="30" customHeight="1" spans="1:7">
       <c r="A49" s="9">
@@ -2930,18 +2988,20 @@
       </c>
       <c r="B49" s="10"/>
       <c r="C49" s="11" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="D49" s="12" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="E49" s="13" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="F49" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="G49" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G49" s="12" t="s">
+        <v>162</v>
+      </c>
     </row>
     <row r="50" ht="30" customHeight="1" spans="1:7">
       <c r="A50" s="14">
@@ -2949,18 +3009,20 @@
       </c>
       <c r="B50" s="15"/>
       <c r="C50" s="16" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="D50" s="17" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="E50" s="18" t="s">
-        <v>160</v>
-      </c>
-      <c r="F50" s="18" t="s">
-        <v>146</v>
-      </c>
-      <c r="G50" s="17"/>
+        <v>165</v>
+      </c>
+      <c r="F50" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G50" s="17" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row r="51" ht="30" customHeight="1" spans="1:7">
       <c r="A51" s="9">
@@ -2968,18 +3030,20 @@
       </c>
       <c r="B51" s="10"/>
       <c r="C51" s="11" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="D51" s="12" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="E51" s="13" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="F51" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="G51" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G51" s="12" t="s">
+        <v>170</v>
+      </c>
     </row>
     <row r="52" ht="30" customHeight="1" spans="1:7">
       <c r="A52" s="14">
@@ -2987,18 +3051,20 @@
       </c>
       <c r="B52" s="15"/>
       <c r="C52" s="16" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="D52" s="17" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="E52" s="18" t="s">
-        <v>163</v>
-      </c>
-      <c r="F52" s="18" t="s">
-        <v>146</v>
-      </c>
-      <c r="G52" s="17"/>
+        <v>169</v>
+      </c>
+      <c r="F52" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G52" s="17" t="s">
+        <v>173</v>
+      </c>
     </row>
     <row r="53" ht="30" customHeight="1" spans="1:7">
       <c r="A53" s="9">
@@ -3006,18 +3072,20 @@
       </c>
       <c r="B53" s="10"/>
       <c r="C53" s="11" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D53" s="12" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="E53" s="13" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="F53" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="G53" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G53" s="12" t="s">
+        <v>177</v>
+      </c>
     </row>
     <row r="54" ht="30" customHeight="1" spans="1:7">
       <c r="A54" s="14">
@@ -3025,18 +3093,20 @@
       </c>
       <c r="B54" s="15"/>
       <c r="C54" s="16" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="D54" s="17" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="E54" s="18" t="s">
-        <v>168</v>
-      </c>
-      <c r="F54" s="18" t="s">
-        <v>146</v>
-      </c>
-      <c r="G54" s="17"/>
+        <v>176</v>
+      </c>
+      <c r="F54" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G54" s="17" t="s">
+        <v>180</v>
+      </c>
     </row>
     <row r="55" ht="30" customHeight="1" spans="1:7">
       <c r="A55" s="9">
@@ -3044,18 +3114,20 @@
       </c>
       <c r="B55" s="10"/>
       <c r="C55" s="11" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="D55" s="12" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="E55" s="13" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="F55" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="G55" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G55" s="12" t="s">
+        <v>184</v>
+      </c>
     </row>
     <row r="56" ht="30" customHeight="1" spans="1:7">
       <c r="A56" s="14">
@@ -3066,15 +3138,17 @@
         <v>77</v>
       </c>
       <c r="D56" s="17" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="E56" s="18" t="s">
-        <v>173</v>
-      </c>
-      <c r="F56" s="18" t="s">
-        <v>146</v>
-      </c>
-      <c r="G56" s="17"/>
+        <v>183</v>
+      </c>
+      <c r="F56" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G56" s="17" t="s">
+        <v>186</v>
+      </c>
     </row>
     <row r="57" ht="30" customHeight="1" spans="1:7">
       <c r="A57" s="9">
@@ -3085,15 +3159,17 @@
         <v>81</v>
       </c>
       <c r="D57" s="12" t="s">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="E57" s="13" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="F57" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="G57" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G57" s="12" t="s">
+        <v>188</v>
+      </c>
     </row>
     <row r="58" ht="30" customHeight="1" spans="1:7">
       <c r="A58" s="14">
@@ -3101,18 +3177,20 @@
       </c>
       <c r="B58" s="15"/>
       <c r="C58" s="16" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="D58" s="17" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="E58" s="18" t="s">
-        <v>178</v>
-      </c>
-      <c r="F58" s="18" t="s">
-        <v>146</v>
-      </c>
-      <c r="G58" s="17"/>
+        <v>191</v>
+      </c>
+      <c r="F58" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G58" s="17" t="s">
+        <v>192</v>
+      </c>
     </row>
     <row r="59" ht="30" customHeight="1" spans="1:7">
       <c r="A59" s="9">
@@ -3120,18 +3198,20 @@
       </c>
       <c r="B59" s="10"/>
       <c r="C59" s="11" t="s">
-        <v>179</v>
+        <v>193</v>
       </c>
       <c r="D59" s="12" t="s">
-        <v>180</v>
+        <v>194</v>
       </c>
       <c r="E59" s="13" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="F59" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="G59" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G59" s="12" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="60" ht="30" customHeight="1" spans="1:7">
       <c r="A60" s="14">
@@ -3142,34 +3222,36 @@
         <v>91</v>
       </c>
       <c r="D60" s="17" t="s">
-        <v>181</v>
+        <v>196</v>
       </c>
       <c r="E60" s="18" t="s">
-        <v>178</v>
-      </c>
-      <c r="F60" s="18" t="s">
-        <v>146</v>
-      </c>
-      <c r="G60" s="17"/>
+        <v>191</v>
+      </c>
+      <c r="F60" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G60" s="17" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="61" ht="30" customHeight="1" spans="1:7">
       <c r="A61" s="9">
         <v>55</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>182</v>
+        <v>197</v>
       </c>
       <c r="C61" s="11" t="s">
-        <v>183</v>
+        <v>198</v>
       </c>
       <c r="D61" s="12" t="s">
-        <v>184</v>
+        <v>199</v>
       </c>
       <c r="E61" s="13" t="s">
-        <v>185</v>
+        <v>200</v>
       </c>
       <c r="F61" s="13" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="G61" s="12"/>
     </row>
@@ -3179,16 +3261,16 @@
       </c>
       <c r="B62" s="15"/>
       <c r="C62" s="16" t="s">
-        <v>186</v>
+        <v>202</v>
       </c>
       <c r="D62" s="17" t="s">
-        <v>187</v>
+        <v>203</v>
       </c>
       <c r="E62" s="18" t="s">
-        <v>188</v>
+        <v>204</v>
       </c>
       <c r="F62" s="18" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="G62" s="17"/>
     </row>
@@ -3198,16 +3280,16 @@
       </c>
       <c r="B63" s="10"/>
       <c r="C63" s="11" t="s">
-        <v>189</v>
+        <v>205</v>
       </c>
       <c r="D63" s="12" t="s">
-        <v>190</v>
+        <v>206</v>
       </c>
       <c r="E63" s="13" t="s">
-        <v>191</v>
+        <v>207</v>
       </c>
       <c r="F63" s="13" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="G63" s="12"/>
     </row>
@@ -3217,16 +3299,16 @@
       </c>
       <c r="B64" s="15"/>
       <c r="C64" s="16" t="s">
-        <v>192</v>
+        <v>208</v>
       </c>
       <c r="D64" s="17" t="s">
-        <v>193</v>
+        <v>209</v>
       </c>
       <c r="E64" s="18" t="s">
-        <v>194</v>
+        <v>210</v>
       </c>
       <c r="F64" s="18" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="G64" s="17"/>
     </row>
@@ -3236,16 +3318,16 @@
       </c>
       <c r="B65" s="10"/>
       <c r="C65" s="11" t="s">
-        <v>195</v>
+        <v>211</v>
       </c>
       <c r="D65" s="12" t="s">
-        <v>196</v>
+        <v>212</v>
       </c>
       <c r="E65" s="13" t="s">
-        <v>197</v>
+        <v>213</v>
       </c>
       <c r="F65" s="13" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="G65" s="12"/>
     </row>
@@ -3255,16 +3337,16 @@
       </c>
       <c r="B66" s="15"/>
       <c r="C66" s="16" t="s">
-        <v>198</v>
+        <v>214</v>
       </c>
       <c r="D66" s="17" t="s">
-        <v>199</v>
+        <v>215</v>
       </c>
       <c r="E66" s="18" t="s">
-        <v>200</v>
+        <v>216</v>
       </c>
       <c r="F66" s="18" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="G66" s="17"/>
     </row>
@@ -3274,16 +3356,16 @@
       </c>
       <c r="B67" s="10"/>
       <c r="C67" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="D67" s="12" t="s">
+        <v>218</v>
+      </c>
+      <c r="E67" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="F67" s="13" t="s">
         <v>201</v>
-      </c>
-      <c r="D67" s="12" t="s">
-        <v>202</v>
-      </c>
-      <c r="E67" s="13" t="s">
-        <v>203</v>
-      </c>
-      <c r="F67" s="13" t="s">
-        <v>146</v>
       </c>
       <c r="G67" s="12"/>
     </row>
@@ -3293,16 +3375,16 @@
       </c>
       <c r="B68" s="15"/>
       <c r="C68" s="16" t="s">
-        <v>204</v>
+        <v>220</v>
       </c>
       <c r="D68" s="17" t="s">
-        <v>205</v>
+        <v>221</v>
       </c>
       <c r="E68" s="18" t="s">
-        <v>206</v>
+        <v>222</v>
       </c>
       <c r="F68" s="18" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="G68" s="17"/>
     </row>
@@ -3312,16 +3394,16 @@
       </c>
       <c r="B69" s="10"/>
       <c r="C69" s="11" t="s">
-        <v>207</v>
+        <v>223</v>
       </c>
       <c r="D69" s="12" t="s">
-        <v>208</v>
+        <v>224</v>
       </c>
       <c r="E69" s="13" t="s">
-        <v>209</v>
+        <v>225</v>
       </c>
       <c r="F69" s="13" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="G69" s="12"/>
     </row>
@@ -3331,16 +3413,16 @@
       </c>
       <c r="B70" s="15"/>
       <c r="C70" s="16" t="s">
-        <v>210</v>
+        <v>226</v>
       </c>
       <c r="D70" s="17" t="s">
-        <v>211</v>
+        <v>227</v>
       </c>
       <c r="E70" s="18" t="s">
-        <v>212</v>
+        <v>228</v>
       </c>
       <c r="F70" s="18" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="G70" s="17"/>
     </row>
@@ -3350,16 +3432,16 @@
       </c>
       <c r="B71" s="10"/>
       <c r="C71" s="11" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="D71" s="12" t="s">
-        <v>214</v>
+        <v>230</v>
       </c>
       <c r="E71" s="13" t="s">
-        <v>215</v>
+        <v>231</v>
       </c>
       <c r="F71" s="13" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="G71" s="12"/>
     </row>
@@ -3369,16 +3451,16 @@
       </c>
       <c r="B72" s="15"/>
       <c r="C72" s="16" t="s">
-        <v>216</v>
+        <v>232</v>
       </c>
       <c r="D72" s="17" t="s">
-        <v>217</v>
+        <v>233</v>
       </c>
       <c r="E72" s="18" t="s">
-        <v>215</v>
+        <v>231</v>
       </c>
       <c r="F72" s="18" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="G72" s="17"/>
     </row>
@@ -3388,16 +3470,16 @@
       </c>
       <c r="B73" s="10"/>
       <c r="C73" s="11" t="s">
-        <v>218</v>
+        <v>234</v>
       </c>
       <c r="D73" s="12" t="s">
-        <v>219</v>
+        <v>235</v>
       </c>
       <c r="E73" s="13" t="s">
-        <v>220</v>
+        <v>236</v>
       </c>
       <c r="F73" s="13" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="G73" s="12"/>
     </row>
@@ -3407,16 +3489,16 @@
       </c>
       <c r="B74" s="15"/>
       <c r="C74" s="16" t="s">
-        <v>221</v>
+        <v>237</v>
       </c>
       <c r="D74" s="17" t="s">
-        <v>222</v>
+        <v>238</v>
       </c>
       <c r="E74" s="18" t="s">
-        <v>220</v>
+        <v>236</v>
       </c>
       <c r="F74" s="18" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="G74" s="17"/>
     </row>
@@ -3426,16 +3508,16 @@
       </c>
       <c r="B75" s="10"/>
       <c r="C75" s="11" t="s">
-        <v>223</v>
+        <v>239</v>
       </c>
       <c r="D75" s="12" t="s">
-        <v>224</v>
+        <v>240</v>
       </c>
       <c r="E75" s="13" t="s">
-        <v>225</v>
+        <v>241</v>
       </c>
       <c r="F75" s="13" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="G75" s="12"/>
     </row>
@@ -3445,16 +3527,16 @@
       </c>
       <c r="B76" s="15"/>
       <c r="C76" s="16" t="s">
-        <v>226</v>
+        <v>242</v>
       </c>
       <c r="D76" s="17" t="s">
-        <v>227</v>
+        <v>243</v>
       </c>
       <c r="E76" s="18" t="s">
-        <v>225</v>
+        <v>241</v>
       </c>
       <c r="F76" s="18" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="G76" s="17"/>
     </row>
@@ -3464,16 +3546,16 @@
       </c>
       <c r="B77" s="10"/>
       <c r="C77" s="11" t="s">
-        <v>228</v>
+        <v>244</v>
       </c>
       <c r="D77" s="12" t="s">
-        <v>229</v>
+        <v>245</v>
       </c>
       <c r="E77" s="13" t="s">
-        <v>225</v>
+        <v>241</v>
       </c>
       <c r="F77" s="13" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="G77" s="12"/>
     </row>
@@ -3483,16 +3565,16 @@
       </c>
       <c r="B78" s="15"/>
       <c r="C78" s="16" t="s">
-        <v>230</v>
+        <v>246</v>
       </c>
       <c r="D78" s="17" t="s">
-        <v>231</v>
+        <v>247</v>
       </c>
       <c r="E78" s="18" t="s">
-        <v>232</v>
+        <v>248</v>
       </c>
       <c r="F78" s="18" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="G78" s="17"/>
     </row>
@@ -3502,16 +3584,16 @@
       </c>
       <c r="B79" s="10"/>
       <c r="C79" s="11" t="s">
-        <v>233</v>
+        <v>249</v>
       </c>
       <c r="D79" s="12" t="s">
-        <v>234</v>
+        <v>250</v>
       </c>
       <c r="E79" s="13" t="s">
-        <v>232</v>
+        <v>248</v>
       </c>
       <c r="F79" s="13" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="G79" s="12"/>
     </row>
@@ -3521,16 +3603,16 @@
       </c>
       <c r="B80" s="15"/>
       <c r="C80" s="16" t="s">
-        <v>235</v>
+        <v>251</v>
       </c>
       <c r="D80" s="17" t="s">
-        <v>236</v>
+        <v>252</v>
       </c>
       <c r="E80" s="18" t="s">
-        <v>237</v>
+        <v>253</v>
       </c>
       <c r="F80" s="18" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="G80" s="17"/>
     </row>
@@ -3540,16 +3622,16 @@
       </c>
       <c r="B81" s="10"/>
       <c r="C81" s="11" t="s">
-        <v>238</v>
+        <v>254</v>
       </c>
       <c r="D81" s="12" t="s">
-        <v>239</v>
+        <v>255</v>
       </c>
       <c r="E81" s="13" t="s">
-        <v>237</v>
+        <v>253</v>
       </c>
       <c r="F81" s="13" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="G81" s="12"/>
     </row>
@@ -3559,16 +3641,16 @@
       </c>
       <c r="B82" s="15"/>
       <c r="C82" s="16" t="s">
-        <v>240</v>
+        <v>256</v>
       </c>
       <c r="D82" s="17" t="s">
-        <v>241</v>
+        <v>257</v>
       </c>
       <c r="E82" s="18" t="s">
-        <v>237</v>
+        <v>253</v>
       </c>
       <c r="F82" s="18" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="G82" s="17"/>
     </row>
@@ -3578,16 +3660,16 @@
       </c>
       <c r="B83" s="10"/>
       <c r="C83" s="11" t="s">
-        <v>242</v>
+        <v>258</v>
       </c>
       <c r="D83" s="12" t="s">
-        <v>243</v>
+        <v>259</v>
       </c>
       <c r="E83" s="13" t="s">
-        <v>237</v>
+        <v>253</v>
       </c>
       <c r="F83" s="13" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="G83" s="12"/>
     </row>
@@ -3597,16 +3679,16 @@
       </c>
       <c r="B84" s="10"/>
       <c r="C84" s="11" t="s">
-        <v>244</v>
+        <v>260</v>
       </c>
       <c r="D84" s="12" t="s">
-        <v>245</v>
+        <v>261</v>
       </c>
       <c r="E84" s="13" t="s">
-        <v>237</v>
+        <v>253</v>
       </c>
       <c r="F84" s="13" t="s">
-        <v>146</v>
+        <v>201</v>
       </c>
       <c r="G84" s="12"/>
     </row>
@@ -3630,7 +3712,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F7:F29 F30:F43 F44:F84">
+    <dataValidation type="list" allowBlank="1" sqref="F7:F84">
       <formula1>"Not Started,In Progress,Done,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3652,73 +3734,73 @@
   <sheetData>
     <row r="1" ht="27.75" customHeight="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>246</v>
+        <v>262</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="3" ht="30" customHeight="1" spans="2:2">
       <c r="B3" s="2" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="2:2">
       <c r="B4" s="2" t="s">
-        <v>248</v>
+        <v>264</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="2:2">
       <c r="B5" s="2" t="s">
-        <v>249</v>
+        <v>265</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="2:2">
       <c r="B6" s="2" t="s">
-        <v>250</v>
+        <v>266</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="2:2">
       <c r="B7" s="2" t="s">
-        <v>251</v>
+        <v>267</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" spans="2:2">
       <c r="B8" s="2" t="s">
-        <v>252</v>
+        <v>268</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" spans="2:2">
       <c r="B9" s="2" t="s">
-        <v>253</v>
+        <v>269</v>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1" spans="2:2">
       <c r="B10" s="2" t="s">
-        <v>254</v>
+        <v>270</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1" spans="2:2">
       <c r="B11" s="2" t="s">
-        <v>255</v>
+        <v>271</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1" spans="2:2">
       <c r="B12" s="2" t="s">
-        <v>256</v>
+        <v>272</v>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1" spans="2:2">
       <c r="B13" s="2" t="s">
-        <v>257</v>
+        <v>273</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1" spans="2:2">
       <c r="B14" s="2" t="s">
-        <v>258</v>
+        <v>274</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1" spans="2:2">
       <c r="B15" s="2" t="s">
-        <v>259</v>
+        <v>275</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add updated checklist and project demo
</commit_message>
<xml_diff>
--- a/checklist.xlsx
+++ b/checklist.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="299">
   <si>
     <t>iNeuBytes  •  45-Day Web Development Internship  -  Intern Checklist</t>
   </si>
@@ -633,7 +633,7 @@
     <t>25-26</t>
   </si>
   <si>
-    <t>Not Started</t>
+    <t>Secured registration and login for Patient, Doctor and Admin.</t>
   </si>
   <si>
     <t>Auth: role-based access control</t>
@@ -645,6 +645,9 @@
     <t>26</t>
   </si>
   <si>
+    <t>Implemented role-based authentication and authorization for Patient, Doctor and Admin.</t>
+  </si>
+  <si>
     <t>Frontend: core pages (HTML/CSS)</t>
   </si>
   <si>
@@ -654,6 +657,9 @@
     <t>27-29</t>
   </si>
   <si>
+    <t>Developed responsive Home, Login/Register, Patient, Doctor, Admin, Appointment, Department and Contact pages.</t>
+  </si>
+  <si>
     <t>Backend: server + secure sessions</t>
   </si>
   <si>
@@ -663,6 +669,9 @@
     <t>30</t>
   </si>
   <si>
+    <t>Implemented Node.js/Express backend with secure JWT-based authentication.</t>
+  </si>
+  <si>
     <t>Backend: database + relationships</t>
   </si>
   <si>
@@ -672,6 +681,9 @@
     <t>30-31</t>
   </si>
   <si>
+    <t>Integrated MongoDB Atlas with related User, Patient, Doctor, Appointment and Department data.</t>
+  </si>
+  <si>
     <t>Backend: RESTful API + CRUD</t>
   </si>
   <si>
@@ -681,6 +693,9 @@
     <t>31-32</t>
   </si>
   <si>
+    <t>Implemented RESTful endpoints with CRUD operations for major modules.</t>
+  </si>
+  <si>
     <t>Backend: security</t>
   </si>
   <si>
@@ -690,6 +705,9 @@
     <t>32</t>
   </si>
   <si>
+    <t>Added password hashing, JWT authentication, role authorization, validation and centralized error handling.</t>
+  </si>
+  <si>
     <t>Patient Dashboard</t>
   </si>
   <si>
@@ -699,6 +717,9 @@
     <t>33</t>
   </si>
   <si>
+    <t>Profile management, appointment booking/history, medical records and notifications.</t>
+  </si>
+  <si>
     <t>Doctor Dashboard</t>
   </si>
   <si>
@@ -708,6 +729,9 @@
     <t>34</t>
   </si>
   <si>
+    <t>Appointment management, patient details, consultation status and profile management.</t>
+  </si>
+  <si>
     <t>Admin Dashboard</t>
   </si>
   <si>
@@ -717,6 +741,9 @@
     <t>35</t>
   </si>
   <si>
+    <t>Management of patients, doctors, departments and appointments with statistics.</t>
+  </si>
+  <si>
     <t>Department management</t>
   </si>
   <si>
@@ -726,12 +753,18 @@
     <t>36</t>
   </si>
   <si>
+    <t>Department creation, management, doctor assignment and department-wise listings.</t>
+  </si>
+  <si>
     <t>Appointment management</t>
   </si>
   <si>
     <t>Book / reschedule / cancel; appointment status management</t>
   </si>
   <si>
+    <t>Booking, management, status updates and appointment history.</t>
+  </si>
+  <si>
     <t>Notification management</t>
   </si>
   <si>
@@ -741,12 +774,18 @@
     <t>37</t>
   </si>
   <si>
+    <t>Implemented notification functionality for appointment/status-related updates.</t>
+  </si>
+  <si>
     <t>Profile management</t>
   </si>
   <si>
     <t>Update profile, change password, upload profile picture</t>
   </si>
   <si>
+    <t>Profile information update and account management.</t>
+  </si>
+  <si>
     <t>Search &amp; reports</t>
   </si>
   <si>
@@ -756,18 +795,27 @@
     <t>38</t>
   </si>
   <si>
+    <t>Implemented search/filtering, dashboard statistics and reporting functionality.</t>
+  </si>
+  <si>
     <t>JS: dynamic features</t>
   </si>
   <si>
     <t>Dynamic booking, dashboard interactions, search/filter, statistics cards, role-based nav, charts (optional)</t>
   </si>
   <si>
+    <t>Dynamic dashboards, booking interactions, search/filtering, role-based navigation and statistics.</t>
+  </si>
+  <si>
     <t>File upload support (optional)</t>
   </si>
   <si>
     <t>Enable file/image uploads where relevant</t>
   </si>
   <si>
+    <t>Implemented relevant profile/file upload functionality.</t>
+  </si>
+  <si>
     <t>Test &amp; debug all modules</t>
   </si>
   <si>
@@ -777,12 +825,21 @@
     <t>39</t>
   </si>
   <si>
+    <t>Tested authentication, CRUD operations, dashboards, responsiveness and major user workflows.</t>
+  </si>
+  <si>
     <t>Deployment (optional)</t>
   </si>
   <si>
     <t>Prepare for deployment, configure env variables, deploy frontend &amp; backend, verify functionality</t>
   </si>
   <si>
+    <t>Not Completed</t>
+  </si>
+  <si>
+    <t>Major Project committed and pushed with project documentation.</t>
+  </si>
+  <si>
     <t>Push Major Project to GitHub</t>
   </si>
   <si>
@@ -798,22 +855,34 @@
     <t>System architecture, database design, methodology, challenges, solutions</t>
   </si>
   <si>
+    <t>Development report completed with architecture, database design, methodology, challenges and solutions.</t>
+  </si>
+  <si>
     <t>Prepare project documentation in Google Doc, Upload in GitHub</t>
   </si>
   <si>
     <t>Installation steps, project structure, database schema, API docs, future enhancements</t>
   </si>
   <si>
+    <t>Installation, project structure, database/API information and future enhancements documented.</t>
+  </si>
+  <si>
     <t>Record project demo video, upload in GitHub</t>
   </si>
   <si>
     <t>Features, responsiveness, overall workflow</t>
   </si>
   <si>
+    <t>Project demonstration video recorded and uploaded.</t>
+  </si>
+  <si>
     <t>Submit Intern Checklist, upload to GitHub</t>
   </si>
   <si>
     <t>overall workflow</t>
+  </si>
+  <si>
+    <t>Internship checklist completed and uploaded to GitHub.</t>
   </si>
   <si>
     <t>Key Rules &amp; Reminders — iNeuBytes VIIP (WBINB20726)</t>
@@ -2062,8 +2131,8 @@
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
       <c r="D4" s="7" t="str">
-        <f>"54 of 78 done   ("&amp;TEXT(54/78,"0%")&amp;" complete)   |   In Progress: 1   |   Blocked: 0"</f>
-        <v>54 of 78 done   (69% complete)   |   In Progress: 1   |   Blocked: 0</v>
+        <f>"78 of 78 done   ("&amp;TEXT(78/78,"0%")&amp;" complete)   |   In Progress: 0  |   Blocked: 0"</f>
+        <v>78 of 78 done   (100% complete)   |   In Progress: 0  |   Blocked: 0</v>
       </c>
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
@@ -3251,9 +3320,11 @@
         <v>200</v>
       </c>
       <c r="F61" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G61" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="G61" s="12"/>
     </row>
     <row r="62" ht="30" customHeight="1" spans="1:7">
       <c r="A62" s="14">
@@ -3269,10 +3340,12 @@
       <c r="E62" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="F62" s="18" t="s">
-        <v>201</v>
-      </c>
-      <c r="G62" s="17"/>
+      <c r="F62" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G62" s="17" t="s">
+        <v>205</v>
+      </c>
     </row>
     <row r="63" ht="30" customHeight="1" spans="1:7">
       <c r="A63" s="9">
@@ -3280,18 +3353,20 @@
       </c>
       <c r="B63" s="10"/>
       <c r="C63" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D63" s="12" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E63" s="13" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F63" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="G63" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G63" s="12" t="s">
+        <v>209</v>
+      </c>
     </row>
     <row r="64" ht="30" customHeight="1" spans="1:7">
       <c r="A64" s="14">
@@ -3299,18 +3374,20 @@
       </c>
       <c r="B64" s="15"/>
       <c r="C64" s="16" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D64" s="17" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E64" s="18" t="s">
-        <v>210</v>
-      </c>
-      <c r="F64" s="18" t="s">
-        <v>201</v>
-      </c>
-      <c r="G64" s="17"/>
+        <v>212</v>
+      </c>
+      <c r="F64" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G64" s="17" t="s">
+        <v>213</v>
+      </c>
     </row>
     <row r="65" ht="30" customHeight="1" spans="1:7">
       <c r="A65" s="9">
@@ -3318,18 +3395,20 @@
       </c>
       <c r="B65" s="10"/>
       <c r="C65" s="11" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="D65" s="12" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="E65" s="13" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F65" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="G65" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G65" s="12" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="66" ht="30" customHeight="1" spans="1:7">
       <c r="A66" s="14">
@@ -3337,18 +3416,20 @@
       </c>
       <c r="B66" s="15"/>
       <c r="C66" s="16" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="D66" s="17" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="E66" s="18" t="s">
-        <v>216</v>
-      </c>
-      <c r="F66" s="18" t="s">
-        <v>201</v>
-      </c>
-      <c r="G66" s="17"/>
+        <v>220</v>
+      </c>
+      <c r="F66" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G66" s="17" t="s">
+        <v>221</v>
+      </c>
     </row>
     <row r="67" ht="30" customHeight="1" spans="1:7">
       <c r="A67" s="9">
@@ -3356,18 +3437,20 @@
       </c>
       <c r="B67" s="10"/>
       <c r="C67" s="11" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="D67" s="12" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="E67" s="13" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="F67" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="G67" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G67" s="12" t="s">
+        <v>225</v>
+      </c>
     </row>
     <row r="68" ht="30" customHeight="1" spans="1:7">
       <c r="A68" s="14">
@@ -3375,18 +3458,20 @@
       </c>
       <c r="B68" s="15"/>
       <c r="C68" s="16" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="D68" s="17" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="E68" s="18" t="s">
-        <v>222</v>
-      </c>
-      <c r="F68" s="18" t="s">
-        <v>201</v>
-      </c>
-      <c r="G68" s="17"/>
+        <v>228</v>
+      </c>
+      <c r="F68" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G68" s="17" t="s">
+        <v>229</v>
+      </c>
     </row>
     <row r="69" ht="30" customHeight="1" spans="1:7">
       <c r="A69" s="9">
@@ -3394,18 +3479,20 @@
       </c>
       <c r="B69" s="10"/>
       <c r="C69" s="11" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="D69" s="12" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="E69" s="13" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="F69" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="G69" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G69" s="12" t="s">
+        <v>233</v>
+      </c>
     </row>
     <row r="70" ht="30" customHeight="1" spans="1:7">
       <c r="A70" s="14">
@@ -3413,18 +3500,20 @@
       </c>
       <c r="B70" s="15"/>
       <c r="C70" s="16" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="D70" s="17" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E70" s="18" t="s">
-        <v>228</v>
-      </c>
-      <c r="F70" s="18" t="s">
-        <v>201</v>
-      </c>
-      <c r="G70" s="17"/>
+        <v>236</v>
+      </c>
+      <c r="F70" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G70" s="12" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="71" ht="30" customHeight="1" spans="1:7">
       <c r="A71" s="9">
@@ -3432,18 +3521,20 @@
       </c>
       <c r="B71" s="10"/>
       <c r="C71" s="11" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="D71" s="12" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="E71" s="13" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
       <c r="F71" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="G71" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G71" s="12" t="s">
+        <v>241</v>
+      </c>
     </row>
     <row r="72" ht="30" customHeight="1" spans="1:7">
       <c r="A72" s="14">
@@ -3451,18 +3542,20 @@
       </c>
       <c r="B72" s="15"/>
       <c r="C72" s="16" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="D72" s="17" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
       <c r="E72" s="18" t="s">
-        <v>231</v>
-      </c>
-      <c r="F72" s="18" t="s">
-        <v>201</v>
-      </c>
-      <c r="G72" s="17"/>
+        <v>240</v>
+      </c>
+      <c r="F72" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G72" s="17" t="s">
+        <v>244</v>
+      </c>
     </row>
     <row r="73" ht="30" customHeight="1" spans="1:7">
       <c r="A73" s="9">
@@ -3470,18 +3563,20 @@
       </c>
       <c r="B73" s="10"/>
       <c r="C73" s="11" t="s">
-        <v>234</v>
+        <v>245</v>
       </c>
       <c r="D73" s="12" t="s">
-        <v>235</v>
+        <v>246</v>
       </c>
       <c r="E73" s="13" t="s">
-        <v>236</v>
+        <v>247</v>
       </c>
       <c r="F73" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="G73" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G73" s="12" t="s">
+        <v>248</v>
+      </c>
     </row>
     <row r="74" ht="30" customHeight="1" spans="1:7">
       <c r="A74" s="14">
@@ -3489,18 +3584,20 @@
       </c>
       <c r="B74" s="15"/>
       <c r="C74" s="16" t="s">
-        <v>237</v>
+        <v>249</v>
       </c>
       <c r="D74" s="17" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="E74" s="18" t="s">
-        <v>236</v>
-      </c>
-      <c r="F74" s="18" t="s">
-        <v>201</v>
-      </c>
-      <c r="G74" s="17"/>
+        <v>247</v>
+      </c>
+      <c r="F74" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G74" s="17" t="s">
+        <v>251</v>
+      </c>
     </row>
     <row r="75" ht="30" customHeight="1" spans="1:7">
       <c r="A75" s="9">
@@ -3508,18 +3605,20 @@
       </c>
       <c r="B75" s="10"/>
       <c r="C75" s="11" t="s">
-        <v>239</v>
+        <v>252</v>
       </c>
       <c r="D75" s="12" t="s">
-        <v>240</v>
+        <v>253</v>
       </c>
       <c r="E75" s="13" t="s">
-        <v>241</v>
+        <v>254</v>
       </c>
       <c r="F75" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="G75" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G75" s="12" t="s">
+        <v>255</v>
+      </c>
     </row>
     <row r="76" ht="30" customHeight="1" spans="1:7">
       <c r="A76" s="14">
@@ -3527,18 +3626,20 @@
       </c>
       <c r="B76" s="15"/>
       <c r="C76" s="16" t="s">
-        <v>242</v>
+        <v>256</v>
       </c>
       <c r="D76" s="17" t="s">
-        <v>243</v>
+        <v>257</v>
       </c>
       <c r="E76" s="18" t="s">
-        <v>241</v>
-      </c>
-      <c r="F76" s="18" t="s">
-        <v>201</v>
-      </c>
-      <c r="G76" s="17"/>
+        <v>254</v>
+      </c>
+      <c r="F76" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G76" s="17" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="77" ht="30" customHeight="1" spans="1:7">
       <c r="A77" s="9">
@@ -3546,18 +3647,20 @@
       </c>
       <c r="B77" s="10"/>
       <c r="C77" s="11" t="s">
-        <v>244</v>
+        <v>259</v>
       </c>
       <c r="D77" s="12" t="s">
-        <v>245</v>
+        <v>260</v>
       </c>
       <c r="E77" s="13" t="s">
-        <v>241</v>
+        <v>254</v>
       </c>
       <c r="F77" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="G77" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G77" s="12" t="s">
+        <v>261</v>
+      </c>
     </row>
     <row r="78" ht="30" customHeight="1" spans="1:7">
       <c r="A78" s="14">
@@ -3565,18 +3668,20 @@
       </c>
       <c r="B78" s="15"/>
       <c r="C78" s="16" t="s">
-        <v>246</v>
+        <v>262</v>
       </c>
       <c r="D78" s="17" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
       <c r="E78" s="18" t="s">
-        <v>248</v>
-      </c>
-      <c r="F78" s="18" t="s">
-        <v>201</v>
-      </c>
-      <c r="G78" s="17"/>
+        <v>264</v>
+      </c>
+      <c r="F78" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G78" s="17" t="s">
+        <v>265</v>
+      </c>
     </row>
     <row r="79" ht="30" customHeight="1" spans="1:7">
       <c r="A79" s="9">
@@ -3584,18 +3689,20 @@
       </c>
       <c r="B79" s="10"/>
       <c r="C79" s="11" t="s">
-        <v>249</v>
+        <v>266</v>
       </c>
       <c r="D79" s="12" t="s">
-        <v>250</v>
+        <v>267</v>
       </c>
       <c r="E79" s="13" t="s">
-        <v>248</v>
+        <v>264</v>
       </c>
       <c r="F79" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="G79" s="12"/>
+        <v>268</v>
+      </c>
+      <c r="G79" s="12" t="s">
+        <v>269</v>
+      </c>
     </row>
     <row r="80" ht="30" customHeight="1" spans="1:7">
       <c r="A80" s="14">
@@ -3603,18 +3710,20 @@
       </c>
       <c r="B80" s="15"/>
       <c r="C80" s="16" t="s">
-        <v>251</v>
+        <v>270</v>
       </c>
       <c r="D80" s="17" t="s">
-        <v>252</v>
+        <v>271</v>
       </c>
       <c r="E80" s="18" t="s">
-        <v>253</v>
-      </c>
-      <c r="F80" s="18" t="s">
-        <v>201</v>
-      </c>
-      <c r="G80" s="17"/>
+        <v>272</v>
+      </c>
+      <c r="F80" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G80" s="17" t="s">
+        <v>269</v>
+      </c>
     </row>
     <row r="81" ht="30" customHeight="1" spans="1:7">
       <c r="A81" s="9">
@@ -3622,18 +3731,20 @@
       </c>
       <c r="B81" s="10"/>
       <c r="C81" s="11" t="s">
-        <v>254</v>
+        <v>273</v>
       </c>
       <c r="D81" s="12" t="s">
-        <v>255</v>
+        <v>274</v>
       </c>
       <c r="E81" s="13" t="s">
-        <v>253</v>
+        <v>272</v>
       </c>
       <c r="F81" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="G81" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G81" s="12" t="s">
+        <v>275</v>
+      </c>
     </row>
     <row r="82" ht="30" customHeight="1" spans="1:7">
       <c r="A82" s="14">
@@ -3641,18 +3752,20 @@
       </c>
       <c r="B82" s="15"/>
       <c r="C82" s="16" t="s">
-        <v>256</v>
+        <v>276</v>
       </c>
       <c r="D82" s="17" t="s">
-        <v>257</v>
+        <v>277</v>
       </c>
       <c r="E82" s="18" t="s">
-        <v>253</v>
-      </c>
-      <c r="F82" s="18" t="s">
-        <v>201</v>
-      </c>
-      <c r="G82" s="17"/>
+        <v>272</v>
+      </c>
+      <c r="F82" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G82" s="17" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="83" ht="30" customHeight="1" spans="1:7">
       <c r="A83" s="9">
@@ -3660,18 +3773,20 @@
       </c>
       <c r="B83" s="10"/>
       <c r="C83" s="11" t="s">
-        <v>258</v>
+        <v>279</v>
       </c>
       <c r="D83" s="12" t="s">
-        <v>259</v>
+        <v>280</v>
       </c>
       <c r="E83" s="13" t="s">
-        <v>253</v>
+        <v>272</v>
       </c>
       <c r="F83" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="G83" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G83" s="12" t="s">
+        <v>281</v>
+      </c>
     </row>
     <row r="84" ht="30.5" customHeight="1" spans="1:7">
       <c r="A84" s="9">
@@ -3679,18 +3794,20 @@
       </c>
       <c r="B84" s="10"/>
       <c r="C84" s="11" t="s">
-        <v>260</v>
+        <v>282</v>
       </c>
       <c r="D84" s="12" t="s">
-        <v>261</v>
+        <v>283</v>
       </c>
       <c r="E84" s="13" t="s">
-        <v>253</v>
+        <v>272</v>
       </c>
       <c r="F84" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="G84" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="G84" s="12" t="s">
+        <v>284</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3712,7 +3829,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F7:F84">
+    <dataValidation type="list" allowBlank="1" sqref="F7:F59 F60:F84">
       <formula1>"Not Started,In Progress,Done,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3734,73 +3851,73 @@
   <sheetData>
     <row r="1" ht="27.75" customHeight="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>262</v>
+        <v>285</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="3" ht="30" customHeight="1" spans="2:2">
       <c r="B3" s="2" t="s">
-        <v>263</v>
+        <v>286</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="2:2">
       <c r="B4" s="2" t="s">
-        <v>264</v>
+        <v>287</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="2:2">
       <c r="B5" s="2" t="s">
-        <v>265</v>
+        <v>288</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="2:2">
       <c r="B6" s="2" t="s">
-        <v>266</v>
+        <v>289</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="2:2">
       <c r="B7" s="2" t="s">
-        <v>267</v>
+        <v>290</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" spans="2:2">
       <c r="B8" s="2" t="s">
-        <v>268</v>
+        <v>291</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" spans="2:2">
       <c r="B9" s="2" t="s">
-        <v>269</v>
+        <v>292</v>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1" spans="2:2">
       <c r="B10" s="2" t="s">
-        <v>270</v>
+        <v>293</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1" spans="2:2">
       <c r="B11" s="2" t="s">
-        <v>271</v>
+        <v>294</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1" spans="2:2">
       <c r="B12" s="2" t="s">
-        <v>272</v>
+        <v>295</v>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1" spans="2:2">
       <c r="B13" s="2" t="s">
-        <v>273</v>
+        <v>296</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1" spans="2:2">
       <c r="B14" s="2" t="s">
-        <v>274</v>
+        <v>297</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1" spans="2:2">
       <c r="B15" s="2" t="s">
-        <v>275</v>
+        <v>298</v>
       </c>
     </row>
   </sheetData>

</xml_diff>